<commit_message>
Add Paid Media tab and confirm the GA4 measurement break
Adds a Paid Media tab built from the keyword-level Google Ads export
(Jan-Jul 2026): monthly totals with CTR, CPC and cost per conversion,
spend, clicks and conversions split by service line, and a corroboration
table lining paid investment up against actual new patients.

The tab resolves the open question on Digital Context. Google Ads clicks
are flat across the period (16,127 in January, 16,944 in July) while GA4
paid-search sessions fall 56%. GA4 sessions per Ads click drop from 0.70
to 0.29, so the traffic did not go away — GA4 stopped recording it.
FLAG 2 is updated from hypothesis to confirmed.

Reported conversions roughly double in June across every campaign at
once, which is flagged on the tab as a probable conversion-tracking
change rather than a performance gain.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MkMRAWDiiUj1quMHQAndcD
</commit_message>
<xml_diff>
--- a/analytics/2026-new-patients-performance-to-budget.xlsx
+++ b/analytics/2026-new-patients-performance-to-budget.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Perf to Budget" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Trends" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Aug Scorecard" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Digital Context" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Paid Media" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Digital Context" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,11 +23,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0);-"/>
     <numFmt numFmtId="167" formatCode="+0.0%;-0.0%;0.0%"/>
+    <numFmt numFmtId="168" formatCode="$#,##0"/>
+    <numFmt numFmtId="169" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -86,7 +89,7 @@
       <sz val="20"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -111,6 +114,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -140,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -191,6 +199,17 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5276,8 +5295,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A28:J28"/>
-    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A4:J4"/>
   </mergeCells>
   <conditionalFormatting sqref="M19:M25">
@@ -6320,6 +6339,1507 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Paid Media — Google Ads, January through July 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source: Monthly_Data_on_Google_Ads_Performance_92.csv, keyword level, 1 Jan - 30 Jul 2026. Blue cells are inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Monthly totals — and the reconciliation against GA4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Total / avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>309482</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>290337</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>429891</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>339799</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>302709</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>341137</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>291599</v>
+      </c>
+      <c r="I6" s="9">
+        <f>SUM(B6:H6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>16127</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>14464</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>21114</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>18136</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>15803</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>17493</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>16944</v>
+      </c>
+      <c r="I7" s="9">
+        <f>SUM(B7:H7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="B8" s="42" t="n">
+        <v>169087.2</v>
+      </c>
+      <c r="C8" s="42" t="n">
+        <v>139994.19</v>
+      </c>
+      <c r="D8" s="42" t="n">
+        <v>283541.48</v>
+      </c>
+      <c r="E8" s="42" t="n">
+        <v>241541.3</v>
+      </c>
+      <c r="F8" s="42" t="n">
+        <v>212153.77</v>
+      </c>
+      <c r="G8" s="42" t="n">
+        <v>279448.97</v>
+      </c>
+      <c r="H8" s="42" t="n">
+        <v>262408.99</v>
+      </c>
+      <c r="I8" s="43">
+        <f>SUM(B8:H8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Reported conversions</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="n">
+        <v>1484.87</v>
+      </c>
+      <c r="C9" s="44" t="n">
+        <v>1128.45</v>
+      </c>
+      <c r="D9" s="44" t="n">
+        <v>1980.88</v>
+      </c>
+      <c r="E9" s="44" t="n">
+        <v>1682.11</v>
+      </c>
+      <c r="F9" s="44" t="n">
+        <v>1454.9</v>
+      </c>
+      <c r="G9" s="44" t="n">
+        <v>3239.1</v>
+      </c>
+      <c r="H9" s="44" t="n">
+        <v>3485.22</v>
+      </c>
+      <c r="I9" s="19">
+        <f>SUM(B9:H9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>GA4 paid-search sessions</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>11258</v>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>5717</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>12612</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>9984</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>5334</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>5937</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>4973</v>
+      </c>
+      <c r="I10" s="9">
+        <f>SUM(B10:H10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Click-through rate</t>
+        </is>
+      </c>
+      <c r="B11" s="45">
+        <f>B7/B6</f>
+        <v/>
+      </c>
+      <c r="C11" s="45">
+        <f>C7/C6</f>
+        <v/>
+      </c>
+      <c r="D11" s="45">
+        <f>D7/D6</f>
+        <v/>
+      </c>
+      <c r="E11" s="45">
+        <f>E7/E6</f>
+        <v/>
+      </c>
+      <c r="F11" s="45">
+        <f>F7/F6</f>
+        <v/>
+      </c>
+      <c r="G11" s="45">
+        <f>G7/G6</f>
+        <v/>
+      </c>
+      <c r="H11" s="45">
+        <f>H7/H6</f>
+        <v/>
+      </c>
+      <c r="I11" s="46">
+        <f>I7/I6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Average cost per click</t>
+        </is>
+      </c>
+      <c r="B12" s="47">
+        <f>B8/B7</f>
+        <v/>
+      </c>
+      <c r="C12" s="47">
+        <f>C8/C7</f>
+        <v/>
+      </c>
+      <c r="D12" s="47">
+        <f>D8/D7</f>
+        <v/>
+      </c>
+      <c r="E12" s="47">
+        <f>E8/E7</f>
+        <v/>
+      </c>
+      <c r="F12" s="47">
+        <f>F8/F7</f>
+        <v/>
+      </c>
+      <c r="G12" s="47">
+        <f>G8/G7</f>
+        <v/>
+      </c>
+      <c r="H12" s="47">
+        <f>H8/H7</f>
+        <v/>
+      </c>
+      <c r="I12" s="48">
+        <f>I8/I7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Cost per reported conversion</t>
+        </is>
+      </c>
+      <c r="B13" s="49">
+        <f>B8/B9</f>
+        <v/>
+      </c>
+      <c r="C13" s="49">
+        <f>C8/C9</f>
+        <v/>
+      </c>
+      <c r="D13" s="49">
+        <f>D8/D9</f>
+        <v/>
+      </c>
+      <c r="E13" s="49">
+        <f>E8/E9</f>
+        <v/>
+      </c>
+      <c r="F13" s="49">
+        <f>F8/F9</f>
+        <v/>
+      </c>
+      <c r="G13" s="49">
+        <f>G8/G9</f>
+        <v/>
+      </c>
+      <c r="H13" s="49">
+        <f>H8/H9</f>
+        <v/>
+      </c>
+      <c r="I13" s="43">
+        <f>I8/I9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>GA4 sessions per Google Ads click</t>
+        </is>
+      </c>
+      <c r="B14" s="50">
+        <f>B10/B7</f>
+        <v/>
+      </c>
+      <c r="C14" s="50">
+        <f>C10/C7</f>
+        <v/>
+      </c>
+      <c r="D14" s="50">
+        <f>D10/D7</f>
+        <v/>
+      </c>
+      <c r="E14" s="50">
+        <f>E10/E7</f>
+        <v/>
+      </c>
+      <c r="F14" s="50">
+        <f>F10/F7</f>
+        <v/>
+      </c>
+      <c r="G14" s="50">
+        <f>G10/G7</f>
+        <v/>
+      </c>
+      <c r="H14" s="50">
+        <f>H10/H7</f>
+        <v/>
+      </c>
+      <c r="I14" s="51">
+        <f>I10/I7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>New patients (all sources)</t>
+        </is>
+      </c>
+      <c r="B15" s="25">
+        <f>Actuals!B12</f>
+        <v/>
+      </c>
+      <c r="C15" s="25">
+        <f>Actuals!C12</f>
+        <v/>
+      </c>
+      <c r="D15" s="25">
+        <f>Actuals!D12</f>
+        <v/>
+      </c>
+      <c r="E15" s="25">
+        <f>Actuals!E12</f>
+        <v/>
+      </c>
+      <c r="F15" s="25">
+        <f>Actuals!F12</f>
+        <v/>
+      </c>
+      <c r="G15" s="25">
+        <f>Actuals!G12</f>
+        <v/>
+      </c>
+      <c r="H15" s="25">
+        <f>Actuals!H12</f>
+        <v/>
+      </c>
+      <c r="I15" s="9">
+        <f>SUM(B15:H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>GA4 sessions per Google Ads click should sit near 0.8-0.9. It falls from 0.70 in January to 0.29 in July while clicks themselves stay flat —</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>that is GA4 losing the ability to record paid visits, not demand going away. This is the confirmation of FLAG 2 on the Digital Context tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Spend by service line</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Service line (from campaign name)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Ortho</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="n">
+        <v>73344.34</v>
+      </c>
+      <c r="C22" s="42" t="n">
+        <v>66874.78</v>
+      </c>
+      <c r="D22" s="42" t="n">
+        <v>176750.4</v>
+      </c>
+      <c r="E22" s="42" t="n">
+        <v>138406.84</v>
+      </c>
+      <c r="F22" s="42" t="n">
+        <v>100328.43</v>
+      </c>
+      <c r="G22" s="42" t="n">
+        <v>124006.65</v>
+      </c>
+      <c r="H22" s="42" t="n">
+        <v>132548.39</v>
+      </c>
+      <c r="I22" s="43">
+        <f>SUM(B22:H22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Spine</t>
+        </is>
+      </c>
+      <c r="B23" s="42" t="n">
+        <v>68091.19</v>
+      </c>
+      <c r="C23" s="42" t="n">
+        <v>42239.6</v>
+      </c>
+      <c r="D23" s="42" t="n">
+        <v>57095.26</v>
+      </c>
+      <c r="E23" s="42" t="n">
+        <v>60736.69</v>
+      </c>
+      <c r="F23" s="42" t="n">
+        <v>66329.98</v>
+      </c>
+      <c r="G23" s="42" t="n">
+        <v>107821.81</v>
+      </c>
+      <c r="H23" s="42" t="n">
+        <v>89047.48</v>
+      </c>
+      <c r="I23" s="43">
+        <f>SUM(B23:H23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Foot</t>
+        </is>
+      </c>
+      <c r="B24" s="42" t="n">
+        <v>6257.23</v>
+      </c>
+      <c r="C24" s="42" t="n">
+        <v>11005.48</v>
+      </c>
+      <c r="D24" s="42" t="n">
+        <v>12673.66</v>
+      </c>
+      <c r="E24" s="42" t="n">
+        <v>12892.2</v>
+      </c>
+      <c r="F24" s="42" t="n">
+        <v>13978.66</v>
+      </c>
+      <c r="G24" s="42" t="n">
+        <v>17093.29</v>
+      </c>
+      <c r="H24" s="42" t="n">
+        <v>14048.26</v>
+      </c>
+      <c r="I24" s="43">
+        <f>SUM(B24:H24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Hand</t>
+        </is>
+      </c>
+      <c r="B25" s="42" t="n">
+        <v>2394.35</v>
+      </c>
+      <c r="C25" s="42" t="n">
+        <v>2227.4</v>
+      </c>
+      <c r="D25" s="42" t="n">
+        <v>4971.03</v>
+      </c>
+      <c r="E25" s="42" t="n">
+        <v>6116.73</v>
+      </c>
+      <c r="F25" s="42" t="n">
+        <v>14117.7</v>
+      </c>
+      <c r="G25" s="42" t="n">
+        <v>18205.08</v>
+      </c>
+      <c r="H25" s="42" t="n">
+        <v>14970.97</v>
+      </c>
+      <c r="I25" s="43">
+        <f>SUM(B25:H25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Brand / other</t>
+        </is>
+      </c>
+      <c r="B26" s="42" t="n">
+        <v>19000.09</v>
+      </c>
+      <c r="C26" s="42" t="n">
+        <v>17646.93</v>
+      </c>
+      <c r="D26" s="42" t="n">
+        <v>32051.13</v>
+      </c>
+      <c r="E26" s="42" t="n">
+        <v>23388.84</v>
+      </c>
+      <c r="F26" s="42" t="n">
+        <v>17399</v>
+      </c>
+      <c r="G26" s="42" t="n">
+        <v>12322.14</v>
+      </c>
+      <c r="H26" s="42" t="n">
+        <v>11793.89</v>
+      </c>
+      <c r="I26" s="43">
+        <f>SUM(B26:H26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B27" s="52">
+        <f>SUM(B22:B26)</f>
+        <v/>
+      </c>
+      <c r="C27" s="52">
+        <f>SUM(C22:C26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="52">
+        <f>SUM(D22:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="52">
+        <f>SUM(E22:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="52">
+        <f>SUM(F22:F26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="52">
+        <f>SUM(G22:G26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="52">
+        <f>SUM(H22:H26)</f>
+        <v/>
+      </c>
+      <c r="I27" s="52">
+        <f>SUM(I22:I26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Campaigns are mapped to service lines by campaign name: Podiatry -&gt; Foot, "Neck, Back, Spine" and "Spine Conditions" -&gt; Spine,</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Orthopedic -&gt; Ortho, Hand -&gt; Hand, and Branded / Doctors / Port Huron / Auto Accident / Canadian Self Pay -&gt; Brand and other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Port Huron is a location campaign covering several lines, so it sits in Brand and other rather than being split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Clicks by service line</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Service line (from campaign name)</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Ortho</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>7959</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>6994</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>11069</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>8548</v>
+      </c>
+      <c r="F35" s="15" t="n">
+        <v>6161</v>
+      </c>
+      <c r="G35" s="15" t="n">
+        <v>6879</v>
+      </c>
+      <c r="H35" s="15" t="n">
+        <v>7115</v>
+      </c>
+      <c r="I35" s="9">
+        <f>SUM(B35:H35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Spine</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n">
+        <v>3243</v>
+      </c>
+      <c r="C36" s="15" t="n">
+        <v>2503</v>
+      </c>
+      <c r="D36" s="15" t="n">
+        <v>3491</v>
+      </c>
+      <c r="E36" s="15" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F36" s="15" t="n">
+        <v>3037</v>
+      </c>
+      <c r="G36" s="15" t="n">
+        <v>3789</v>
+      </c>
+      <c r="H36" s="15" t="n">
+        <v>3222</v>
+      </c>
+      <c r="I36" s="9">
+        <f>SUM(B36:H36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Foot</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n">
+        <v>700</v>
+      </c>
+      <c r="C37" s="15" t="n">
+        <v>1117</v>
+      </c>
+      <c r="D37" s="15" t="n">
+        <v>1285</v>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>1172</v>
+      </c>
+      <c r="F37" s="15" t="n">
+        <v>1149</v>
+      </c>
+      <c r="G37" s="15" t="n">
+        <v>1266</v>
+      </c>
+      <c r="H37" s="15" t="n">
+        <v>1223</v>
+      </c>
+      <c r="I37" s="9">
+        <f>SUM(B37:H37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Hand</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="n">
+        <v>686</v>
+      </c>
+      <c r="C38" s="15" t="n">
+        <v>604</v>
+      </c>
+      <c r="D38" s="15" t="n">
+        <v>1257</v>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>1169</v>
+      </c>
+      <c r="F38" s="15" t="n">
+        <v>1912</v>
+      </c>
+      <c r="G38" s="15" t="n">
+        <v>2348</v>
+      </c>
+      <c r="H38" s="15" t="n">
+        <v>2093</v>
+      </c>
+      <c r="I38" s="9">
+        <f>SUM(B38:H38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Brand / other</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="n">
+        <v>3539</v>
+      </c>
+      <c r="C39" s="15" t="n">
+        <v>3246</v>
+      </c>
+      <c r="D39" s="15" t="n">
+        <v>4012</v>
+      </c>
+      <c r="E39" s="15" t="n">
+        <v>4047</v>
+      </c>
+      <c r="F39" s="15" t="n">
+        <v>3544</v>
+      </c>
+      <c r="G39" s="15" t="n">
+        <v>3211</v>
+      </c>
+      <c r="H39" s="15" t="n">
+        <v>3291</v>
+      </c>
+      <c r="I39" s="9">
+        <f>SUM(B39:H39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B40" s="11">
+        <f>SUM(B35:B39)</f>
+        <v/>
+      </c>
+      <c r="C40" s="11">
+        <f>SUM(C35:C39)</f>
+        <v/>
+      </c>
+      <c r="D40" s="11">
+        <f>SUM(D35:D39)</f>
+        <v/>
+      </c>
+      <c r="E40" s="11">
+        <f>SUM(E35:E39)</f>
+        <v/>
+      </c>
+      <c r="F40" s="11">
+        <f>SUM(F35:F39)</f>
+        <v/>
+      </c>
+      <c r="G40" s="11">
+        <f>SUM(G35:G39)</f>
+        <v/>
+      </c>
+      <c r="H40" s="11">
+        <f>SUM(H35:H39)</f>
+        <v/>
+      </c>
+      <c r="I40" s="11">
+        <f>SUM(I35:I39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Reported conversions by service line</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Service line (from campaign name)</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Ortho</t>
+        </is>
+      </c>
+      <c r="B44" s="44" t="n">
+        <v>730.89</v>
+      </c>
+      <c r="C44" s="44" t="n">
+        <v>487.45</v>
+      </c>
+      <c r="D44" s="44" t="n">
+        <v>885.51</v>
+      </c>
+      <c r="E44" s="44" t="n">
+        <v>757.78</v>
+      </c>
+      <c r="F44" s="44" t="n">
+        <v>549.11</v>
+      </c>
+      <c r="G44" s="44" t="n">
+        <v>1091.87</v>
+      </c>
+      <c r="H44" s="44" t="n">
+        <v>1330.7</v>
+      </c>
+      <c r="I44" s="19">
+        <f>SUM(B44:H44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Spine</t>
+        </is>
+      </c>
+      <c r="B45" s="44" t="n">
+        <v>216.06</v>
+      </c>
+      <c r="C45" s="44" t="n">
+        <v>115.82</v>
+      </c>
+      <c r="D45" s="44" t="n">
+        <v>221.03</v>
+      </c>
+      <c r="E45" s="44" t="n">
+        <v>192.65</v>
+      </c>
+      <c r="F45" s="44" t="n">
+        <v>162.94</v>
+      </c>
+      <c r="G45" s="44" t="n">
+        <v>418.47</v>
+      </c>
+      <c r="H45" s="44" t="n">
+        <v>373.67</v>
+      </c>
+      <c r="I45" s="19">
+        <f>SUM(B45:H45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Foot</t>
+        </is>
+      </c>
+      <c r="B46" s="44" t="n">
+        <v>44.03</v>
+      </c>
+      <c r="C46" s="44" t="n">
+        <v>60.99</v>
+      </c>
+      <c r="D46" s="44" t="n">
+        <v>88.18000000000001</v>
+      </c>
+      <c r="E46" s="44" t="n">
+        <v>80.14</v>
+      </c>
+      <c r="F46" s="44" t="n">
+        <v>67.38</v>
+      </c>
+      <c r="G46" s="44" t="n">
+        <v>153.29</v>
+      </c>
+      <c r="H46" s="44" t="n">
+        <v>132.56</v>
+      </c>
+      <c r="I46" s="19">
+        <f>SUM(B46:H46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Hand</t>
+        </is>
+      </c>
+      <c r="B47" s="44" t="n">
+        <v>78.98</v>
+      </c>
+      <c r="C47" s="44" t="n">
+        <v>40</v>
+      </c>
+      <c r="D47" s="44" t="n">
+        <v>140.57</v>
+      </c>
+      <c r="E47" s="44" t="n">
+        <v>139.82</v>
+      </c>
+      <c r="F47" s="44" t="n">
+        <v>212.47</v>
+      </c>
+      <c r="G47" s="44" t="n">
+        <v>320.05</v>
+      </c>
+      <c r="H47" s="44" t="n">
+        <v>355.16</v>
+      </c>
+      <c r="I47" s="19">
+        <f>SUM(B47:H47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Brand / other</t>
+        </is>
+      </c>
+      <c r="B48" s="44" t="n">
+        <v>414.91</v>
+      </c>
+      <c r="C48" s="44" t="n">
+        <v>424.19</v>
+      </c>
+      <c r="D48" s="44" t="n">
+        <v>645.59</v>
+      </c>
+      <c r="E48" s="44" t="n">
+        <v>511.72</v>
+      </c>
+      <c r="F48" s="44" t="n">
+        <v>463</v>
+      </c>
+      <c r="G48" s="44" t="n">
+        <v>1255.42</v>
+      </c>
+      <c r="H48" s="44" t="n">
+        <v>1293.13</v>
+      </c>
+      <c r="I48" s="19">
+        <f>SUM(B48:H48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B49" s="20">
+        <f>SUM(B44:B48)</f>
+        <v/>
+      </c>
+      <c r="C49" s="20">
+        <f>SUM(C44:C48)</f>
+        <v/>
+      </c>
+      <c r="D49" s="20">
+        <f>SUM(D44:D48)</f>
+        <v/>
+      </c>
+      <c r="E49" s="20">
+        <f>SUM(E44:E48)</f>
+        <v/>
+      </c>
+      <c r="F49" s="20">
+        <f>SUM(F44:F48)</f>
+        <v/>
+      </c>
+      <c r="G49" s="20">
+        <f>SUM(G44:G48)</f>
+        <v/>
+      </c>
+      <c r="H49" s="20">
+        <f>SUM(H44:H48)</f>
+        <v/>
+      </c>
+      <c r="I49" s="20">
+        <f>SUM(I44:I48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>CAUTION: reported conversions roughly double in June across EVERY service line and nearly every campaign at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>A genuine performance gain does not arrive uniformly across unrelated campaigns in the same month. Treat June and July</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>conversion counts, and any cost-per-conversion built from them, as not comparable to January through May until the</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>conversion-action configuration change is confirmed with the paid agency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Does paid investment show up in actual new patients?</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Service line</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Spend Jan-26</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Spend Jul-26</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Spend change</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Clicks change</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>New patients Jan-26</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>New patients Jul-26</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>New patient change</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>YTD attainment vs budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Ortho</t>
+        </is>
+      </c>
+      <c r="B58" s="49">
+        <f>B22</f>
+        <v/>
+      </c>
+      <c r="C58" s="49">
+        <f>H22</f>
+        <v/>
+      </c>
+      <c r="D58" s="29">
+        <f>H22/B22-1</f>
+        <v/>
+      </c>
+      <c r="E58" s="29">
+        <f>H35/B35-1</f>
+        <v/>
+      </c>
+      <c r="F58" s="32">
+        <f>Actuals!B5</f>
+        <v/>
+      </c>
+      <c r="G58" s="32">
+        <f>Actuals!H5</f>
+        <v/>
+      </c>
+      <c r="H58" s="29">
+        <f>Actuals!H5/Actuals!B5-1</f>
+        <v/>
+      </c>
+      <c r="I58" s="23">
+        <f>'Perf to Budget'!I36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Spine</t>
+        </is>
+      </c>
+      <c r="B59" s="49">
+        <f>B23</f>
+        <v/>
+      </c>
+      <c r="C59" s="49">
+        <f>H23</f>
+        <v/>
+      </c>
+      <c r="D59" s="29">
+        <f>H23/B23-1</f>
+        <v/>
+      </c>
+      <c r="E59" s="29">
+        <f>H36/B36-1</f>
+        <v/>
+      </c>
+      <c r="F59" s="32">
+        <f>Actuals!B6</f>
+        <v/>
+      </c>
+      <c r="G59" s="32">
+        <f>Actuals!H6</f>
+        <v/>
+      </c>
+      <c r="H59" s="29">
+        <f>Actuals!H6/Actuals!B6-1</f>
+        <v/>
+      </c>
+      <c r="I59" s="23">
+        <f>'Perf to Budget'!I37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Foot</t>
+        </is>
+      </c>
+      <c r="B60" s="49">
+        <f>B24</f>
+        <v/>
+      </c>
+      <c r="C60" s="49">
+        <f>H24</f>
+        <v/>
+      </c>
+      <c r="D60" s="29">
+        <f>H24/B24-1</f>
+        <v/>
+      </c>
+      <c r="E60" s="29">
+        <f>H37/B37-1</f>
+        <v/>
+      </c>
+      <c r="F60" s="32">
+        <f>Actuals!B8</f>
+        <v/>
+      </c>
+      <c r="G60" s="32">
+        <f>Actuals!H8</f>
+        <v/>
+      </c>
+      <c r="H60" s="29">
+        <f>Actuals!H8/Actuals!B8-1</f>
+        <v/>
+      </c>
+      <c r="I60" s="23">
+        <f>'Perf to Budget'!I39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>Hand</t>
+        </is>
+      </c>
+      <c r="B61" s="49">
+        <f>B25</f>
+        <v/>
+      </c>
+      <c r="C61" s="49">
+        <f>H25</f>
+        <v/>
+      </c>
+      <c r="D61" s="29">
+        <f>H25/B25-1</f>
+        <v/>
+      </c>
+      <c r="E61" s="29">
+        <f>H38/B38-1</f>
+        <v/>
+      </c>
+      <c r="F61" s="32">
+        <f>Actuals!B9</f>
+        <v/>
+      </c>
+      <c r="G61" s="32">
+        <f>Actuals!H9</f>
+        <v/>
+      </c>
+      <c r="H61" s="29">
+        <f>Actuals!H9/Actuals!B9-1</f>
+        <v/>
+      </c>
+      <c r="I61" s="23">
+        <f>'Perf to Budget'!I40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Foot maps to the Podiatry campaigns; the EMR service line is "Foot". Spend and click changes are January versus July.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>This is corroboration, not attribution. The EMR export carries no source field, so no new patient here is proven to have come from paid search.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A56:J56"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A42:J42"/>
+    <mergeCell ref="A33:J33"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6343,10 +7863,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Directional only. GA4 measures website behaviour; it does not attribute new patients. Read the data-quality flags first.</t>
-        </is>
-      </c>
-    </row>
+          <t>Directional only. GA4 measures website behaviour; it does not attribute new patients. See the Paid Media tab for the GA4 reconciliation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -6371,21 +7892,21 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>FLAG 2  Sessions step down about 50% from late April onward and stay there — and the drop hits every channel at once, including</t>
+          <t>FLAG 2  CONFIRMED. Sessions step down about 50% from late April and stay there, across every channel at once. Google Ads</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Direct and Organic. A simultaneous, uniform, all-channel halving is the signature of a tracking or consent change, not of a</t>
+          <t xml:space="preserve">        clicks over the same months are flat (16,127 in January, 16,944 in July), and GA4 sessions per Ads click fall from</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        media decision. Verify against Google Search Console clicks and Google Ads before treating any May-July web number as real.</t>
+          <t xml:space="preserve">        0.70 to 0.29. The traffic did not go away; GA4 stopped recording it. Fix the tagging before using any May-July web number.</t>
         </is>
       </c>
     </row>
@@ -6417,6 +7938,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Attribute the GA4 session drop to the site consent/opt-out widget
SHP added an opt-out widget to the website, which is the cause of the
late-April step down in GA4 sessions. FLAG 2 on Digital Context is
restated from "tracking break, verify" to explained, and two flags are
added: the implied ~71% loss is well above a typical consent banner, so
the widget may be denying analytics by default or firing before the
visitor chooses; and the 18 Feb - 1 Mar blackout predates the widget and
remains unexplained.

Also records the working rule while GA4 is unreliable: use Google Ads
and Search Console clicks for traffic volume, and read GA4 as behaviour
among consented visitors only.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MkMRAWDiiUj1quMHQAndcD
</commit_message>
<xml_diff>
--- a/analytics/2026-new-patients-performance-to-budget.xlsx
+++ b/analytics/2026-new-patients-performance-to-budget.xlsx
@@ -7840,7 +7840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7892,21 +7892,21 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>FLAG 2  CONFIRMED. Sessions step down about 50% from late April and stay there, across every channel at once. Google Ads</t>
+          <t>FLAG 2  EXPLAINED. Sessions step down about 50% from late April and stay there, across every channel at once. SHP added a</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        clicks over the same months are flat (16,127 in January, 16,944 in July), and GA4 sessions per Ads click fall from</t>
+          <t xml:space="preserve">        consent / opt-out widget to the website, which is the cause. Google Ads clicks over the same months are flat (16,127 in</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">        0.70 to 0.29. The traffic did not go away; GA4 stopped recording it. Fix the tagging before using any May-July web number.</t>
+          <t xml:space="preserve">        January, 16,944 in July) while GA4 sessions per Ads click fall 0.70 -&gt; 0.29. Traffic did not fall; consented measurement did.</t>
         </is>
       </c>
     </row>
@@ -7927,270 +7927,132 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Bottom line: patient volume rose every month while measured web sessions fell by half. At least one of those two series is wrong,</t>
+          <t>FLAG 4  A consent / opt-out widget was added to the site. From late April GA4 records only about 29% of the visits Google Ads bills</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>and the patient data — counted from the EMR — is the one to trust.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
+          <t xml:space="preserve">        for, against roughly 70% in January. If that were purely visitors choosing to opt out it would mean a ~71% opt-out rate, which</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        is far above the 10-30% typical of a consent banner. Check whether the widget denies analytics by default or fires before the</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        visitor has chosen, rather than only on an explicit opt-out. Either way GA4 is now a sample, not a census.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>FLAG 5  The widget does not explain the 18 Feb - 1 Mar blackout, which predates it. That remains a separate, unexplained gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Bottom line: patient volume rose every month while measured web sessions fell by half. The web series is the incomplete one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Until GA4 is re-baselined, use Google Ads clicks and Search Console clicks as the measure of traffic volume, and treat GA4 as</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>a directional read on behaviour among consented visitors only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>GA4 monthly summary</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Sessions</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Paid search sessions</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Organic search sessions</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Direct sessions</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Key events</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>New patients</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>New patients per 1,000 sessions</t>
         </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Jan-26</t>
-        </is>
-      </c>
-      <c r="B17" s="15" t="n">
-        <v>21619</v>
-      </c>
-      <c r="C17" s="15" t="n">
-        <v>11258</v>
-      </c>
-      <c r="D17" s="15" t="n">
-        <v>6653</v>
-      </c>
-      <c r="E17" s="15" t="n">
-        <v>2482</v>
-      </c>
-      <c r="F17" s="15" t="n">
-        <v>3595</v>
-      </c>
-      <c r="G17" s="25">
-        <f>Actuals!B12</f>
-        <v/>
-      </c>
-      <c r="H17" s="28">
-        <f>G17/B17*1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Feb-26</t>
-        </is>
-      </c>
-      <c r="B18" s="15" t="n">
-        <v>10893</v>
-      </c>
-      <c r="C18" s="15" t="n">
-        <v>5717</v>
-      </c>
-      <c r="D18" s="15" t="n">
-        <v>3499</v>
-      </c>
-      <c r="E18" s="15" t="n">
-        <v>1186</v>
-      </c>
-      <c r="F18" s="15" t="n">
-        <v>1774</v>
-      </c>
-      <c r="G18" s="25">
-        <f>Actuals!C12</f>
-        <v/>
-      </c>
-      <c r="H18" s="28">
-        <f>G18/B18*1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Mar-26</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="n">
-        <v>21896</v>
-      </c>
-      <c r="C19" s="15" t="n">
-        <v>12612</v>
-      </c>
-      <c r="D19" s="15" t="n">
-        <v>6163</v>
-      </c>
-      <c r="E19" s="15" t="n">
-        <v>2145</v>
-      </c>
-      <c r="F19" s="15" t="n">
-        <v>3298</v>
-      </c>
-      <c r="G19" s="25">
-        <f>Actuals!D12</f>
-        <v/>
-      </c>
-      <c r="H19" s="28">
-        <f>G19/B19*1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Apr-26</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="n">
-        <v>17967</v>
-      </c>
-      <c r="C20" s="15" t="n">
-        <v>9984</v>
-      </c>
-      <c r="D20" s="15" t="n">
-        <v>5264</v>
-      </c>
-      <c r="E20" s="15" t="n">
-        <v>1717</v>
-      </c>
-      <c r="F20" s="15" t="n">
-        <v>2637</v>
-      </c>
-      <c r="G20" s="25">
-        <f>Actuals!E12</f>
-        <v/>
-      </c>
-      <c r="H20" s="28">
-        <f>G20/B20*1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>May-26</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="n">
-        <v>9335</v>
-      </c>
-      <c r="C21" s="15" t="n">
-        <v>5334</v>
-      </c>
-      <c r="D21" s="15" t="n">
-        <v>3027</v>
-      </c>
-      <c r="E21" s="15" t="n">
-        <v>717</v>
-      </c>
-      <c r="F21" s="15" t="n">
-        <v>896</v>
-      </c>
-      <c r="G21" s="25">
-        <f>Actuals!F12</f>
-        <v/>
-      </c>
-      <c r="H21" s="28">
-        <f>G21/B21*1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Jun-26</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="n">
-        <v>10086</v>
-      </c>
-      <c r="C22" s="15" t="n">
-        <v>5937</v>
-      </c>
-      <c r="D22" s="15" t="n">
-        <v>3209</v>
-      </c>
-      <c r="E22" s="15" t="n">
-        <v>669</v>
-      </c>
-      <c r="F22" s="15" t="n">
-        <v>2177</v>
-      </c>
-      <c r="G22" s="25">
-        <f>Actuals!G12</f>
-        <v/>
-      </c>
-      <c r="H22" s="28">
-        <f>G22/B22*1000</f>
-        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Jul-26</t>
+          <t>Jan-26</t>
         </is>
       </c>
       <c r="B23" s="15" t="n">
-        <v>8784</v>
+        <v>21619</v>
       </c>
       <c r="C23" s="15" t="n">
-        <v>4973</v>
+        <v>11258</v>
       </c>
       <c r="D23" s="15" t="n">
-        <v>2768</v>
+        <v>6653</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>594</v>
+        <v>2482</v>
       </c>
       <c r="F23" s="15" t="n">
-        <v>10398</v>
+        <v>3595</v>
       </c>
       <c r="G23" s="25">
-        <f>Actuals!H12</f>
+        <f>Actuals!B12</f>
         <v/>
       </c>
       <c r="H23" s="28">
@@ -8198,22 +8060,202 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>10893</v>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>5717</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>3499</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>1186</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>1774</v>
+      </c>
+      <c r="G24" s="25">
+        <f>Actuals!C12</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>G24/B24*1000</f>
+        <v/>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>21896</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>12612</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>6163</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>2145</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>3298</v>
+      </c>
+      <c r="G25" s="25">
+        <f>Actuals!D12</f>
+        <v/>
+      </c>
+      <c r="H25" s="28">
+        <f>G25/B25*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
+        <v>17967</v>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>9984</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>5264</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>1717</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>2637</v>
+      </c>
+      <c r="G26" s="25">
+        <f>Actuals!E12</f>
+        <v/>
+      </c>
+      <c r="H26" s="28">
+        <f>G26/B26*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>9335</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>5334</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>3027</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>717</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>896</v>
+      </c>
+      <c r="G27" s="25">
+        <f>Actuals!F12</f>
+        <v/>
+      </c>
+      <c r="H27" s="28">
+        <f>G27/B27*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="n">
+        <v>10086</v>
+      </c>
+      <c r="C28" s="15" t="n">
+        <v>5937</v>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>3209</v>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>669</v>
+      </c>
+      <c r="F28" s="15" t="n">
+        <v>2177</v>
+      </c>
+      <c r="G28" s="25">
+        <f>Actuals!G12</f>
+        <v/>
+      </c>
+      <c r="H28" s="28">
+        <f>G28/B28*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>8784</v>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>4973</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>2768</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>594</v>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>10398</v>
+      </c>
+      <c r="G29" s="25">
+        <f>Actuals!H12</f>
+        <v/>
+      </c>
+      <c r="H29" s="28">
+        <f>G29/B29*1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Source: GA4 property 370514163, sessionDefaultChannelGroup by yearMonth, pulled 2026-07-30. July covers 1-29 July only.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>"New patients per 1,000 sessions" is a ratio of two independent series, not a conversion rate. It rises sharply after April because</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>the denominator collapsed, which is exactly what FLAG 2 says not to trust.</t>
         </is>
@@ -8221,8 +8263,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A15:I15"/>
     <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A21:I21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Expense to Budget tab from the 2026 marketing expense plan
Compares Google Ads actual spend against the plan in
Marketing_Expense_Budget_2026.xlsx: $1,588,176 spent Jan-Jul against a
$1,285,000 budget, 23.6% over, with the overage concentrated from March
onward. Google Ads is 64% of the annual OpEx budget, so its variance
drives the plan.

No other expense line has actual spend data, so those are shown as plan
only and explicitly marked unverified rather than assumed on budget.

Also records defects found in the source budget model: the Patient_ROI
tab returns #REF!/#VALUE! throughout, the Summary tab's CPA, ROI,
forecast and gap figures are consequently unusable, Summary reports
annual CapEx as 0 against a $208,000 plan, and the Social_Annual input
disagrees with the OpEx schedule by $504,000.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MkMRAWDiiUj1quMHQAndcD
</commit_message>
<xml_diff>
--- a/analytics/2026-new-patients-performance-to-budget.xlsx
+++ b/analytics/2026-new-patients-performance-to-budget.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Trends" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Aug Scorecard" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Paid Media" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Digital Context" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Expense to Budget" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Digital Context" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,13 +24,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0);-"/>
     <numFmt numFmtId="167" formatCode="+0.0%;-0.0%;0.0%"/>
     <numFmt numFmtId="168" formatCode="$#,##0"/>
     <numFmt numFmtId="169" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="170" formatCode="$#,##0;($#,##0);-"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -148,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -210,6 +212,24 @@
     <xf numFmtId="2" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7840,6 +7860,588 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Marketing Expense to Budget — January through July 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Budget from Marketing_Expense_Budget_2026.xlsx. Only Google Ads has verified actuals; every other line is plan, not spend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Google Ads — the only line with verified actual spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>YTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="B6" s="53" t="n">
+        <v>165000</v>
+      </c>
+      <c r="C6" s="53" t="n">
+        <v>165000</v>
+      </c>
+      <c r="D6" s="53" t="n">
+        <v>185000</v>
+      </c>
+      <c r="E6" s="53" t="n">
+        <v>185000</v>
+      </c>
+      <c r="F6" s="53" t="n">
+        <v>185000</v>
+      </c>
+      <c r="G6" s="53" t="n">
+        <v>200000</v>
+      </c>
+      <c r="H6" s="53" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I6" s="43">
+        <f>SUM(B6:H6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Actual spend</t>
+        </is>
+      </c>
+      <c r="B7" s="53" t="n">
+        <v>169087.2</v>
+      </c>
+      <c r="C7" s="53" t="n">
+        <v>139994.19</v>
+      </c>
+      <c r="D7" s="53" t="n">
+        <v>283541.48</v>
+      </c>
+      <c r="E7" s="53" t="n">
+        <v>241541.3</v>
+      </c>
+      <c r="F7" s="53" t="n">
+        <v>212153.77</v>
+      </c>
+      <c r="G7" s="53" t="n">
+        <v>279448.97</v>
+      </c>
+      <c r="H7" s="53" t="n">
+        <v>262408.99</v>
+      </c>
+      <c r="I7" s="43">
+        <f>SUM(B7:H7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Variance (over / under)</t>
+        </is>
+      </c>
+      <c r="B8" s="54">
+        <f>B7-B6</f>
+        <v/>
+      </c>
+      <c r="C8" s="54">
+        <f>C7-C6</f>
+        <v/>
+      </c>
+      <c r="D8" s="54">
+        <f>D7-D6</f>
+        <v/>
+      </c>
+      <c r="E8" s="54">
+        <f>E7-E6</f>
+        <v/>
+      </c>
+      <c r="F8" s="54">
+        <f>F7-F6</f>
+        <v/>
+      </c>
+      <c r="G8" s="54">
+        <f>G7-G6</f>
+        <v/>
+      </c>
+      <c r="H8" s="54">
+        <f>H7-H6</f>
+        <v/>
+      </c>
+      <c r="I8" s="54">
+        <f>I7-I6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Variance %</t>
+        </is>
+      </c>
+      <c r="B9" s="31">
+        <f>B7/B6-1</f>
+        <v/>
+      </c>
+      <c r="C9" s="31">
+        <f>C7/C6-1</f>
+        <v/>
+      </c>
+      <c r="D9" s="31">
+        <f>D7/D6-1</f>
+        <v/>
+      </c>
+      <c r="E9" s="31">
+        <f>E7/E6-1</f>
+        <v/>
+      </c>
+      <c r="F9" s="31">
+        <f>F7/F6-1</f>
+        <v/>
+      </c>
+      <c r="G9" s="31">
+        <f>G7/G6-1</f>
+        <v/>
+      </c>
+      <c r="H9" s="31">
+        <f>H7/H6-1</f>
+        <v/>
+      </c>
+      <c r="I9" s="31">
+        <f>I7/I6-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>July actual covers 1-30 July only (the export was pulled 30 July), so the July overspend is understated by roughly one day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Google Ads is 64% of the annual OpEx budget ($2,240,000 of $3,485,000), so its variance dominates the whole plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Total marketing budget — plan versus what can be verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Jan-Jul budget</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Jan-Jul actual</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Variance %</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Status of the actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Paid Search - Google</t>
+        </is>
+      </c>
+      <c r="B16" s="53" t="n">
+        <v>1285000</v>
+      </c>
+      <c r="C16" s="55">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="D16" s="56">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+      <c r="E16" s="29">
+        <f>C16/B16-1</f>
+        <v/>
+      </c>
+      <c r="F16" s="36" t="inlineStr">
+        <is>
+          <t>Verified from the Google Ads export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>All other OpEx lines</t>
+        </is>
+      </c>
+      <c r="B17" s="53" t="n">
+        <v>720416.83</v>
+      </c>
+      <c r="C17" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="36" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED. No invoice or spend data supplied — budget shown as a placeholder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>CapEx plan</t>
+        </is>
+      </c>
+      <c r="B18" s="53" t="n">
+        <v>158000</v>
+      </c>
+      <c r="C18" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D18" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="36" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED. No spend data supplied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL Jan-Jul plan</t>
+        </is>
+      </c>
+      <c r="B19" s="52">
+        <f>SUM(B16:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="58" t="n"/>
+      <c r="D19" s="58" t="n"/>
+      <c r="E19" s="58" t="n"/>
+      <c r="F19" s="59" t="inlineStr">
+        <is>
+          <t>Cannot be closed out until the other lines are supplied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>If every non-Google line lands exactly on plan, Jan-Jul marketing OpEx is $2,308,593 against a $2,005,417 budget — 15.1% over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>At the July spend rate, Google Ads finishes 2026 at roughly $2,900,000 against a $2,240,000 full-year budget, about 30% over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Why the overspend happened — the CPA assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Assumption in the budget model</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Paid-search cost per new patient</t>
+        </is>
+      </c>
+      <c r="B26" s="60" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="C26" s="61">
+        <f>I7/Actuals!N12</f>
+        <v/>
+      </c>
+      <c r="D26" s="40" t="inlineStr">
+        <is>
+          <t>Actual divides ALL Google spend by ALL new patients from every source, so it flatters paid search and is still 2x the plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>New patients (annual)</t>
+        </is>
+      </c>
+      <c r="B27" s="60" t="inlineStr">
+        <is>
+          <t>14,400</t>
+        </is>
+      </c>
+      <c r="C27" s="62">
+        <f>Trends!F36</f>
+        <v/>
+      </c>
+      <c r="D27" s="40" t="inlineStr">
+        <is>
+          <t>Full-year projection at the current run rate, from the Trends tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Blended revenue per new patient</t>
+        </is>
+      </c>
+      <c r="B28" s="60" t="inlineStr">
+        <is>
+          <t>$650</t>
+        </is>
+      </c>
+      <c r="C28" s="62" t="inlineStr">
+        <is>
+          <t>not verified</t>
+        </is>
+      </c>
+      <c r="D28" s="40" t="inlineStr">
+        <is>
+          <t>Finance owns this; no actual supplied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>The model derives spend from CPA. A $105 planned CPA against a real cost around double it is the arithmetic reason spend ran over</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>while patient volume ran under. Re-baselining that single input matters more than trimming any individual line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Errors found in the source budget model — fix before this plan is used again</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>The Patient_ROI tab is broken: every row returns #REF! or #VALUE!. It has produced no usable CPA or ROI number all year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>The Summary tab therefore shows #VALUE! for New Patients Forecast, Gap To Goal, Blended CPA, Direct ROI, and the B2C / PL splits —</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>which are exactly the board-facing figures the tab exists to report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Summary!B9 "Total CapEx (Annual)" reads 0, while the CapEx_Plan tab totals $208,000. The Summary understates capital spend by $208,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Inputs!B12 Social_Annual is $720,000, but OpEx_Monthly carries social at $18,000/month = $216,000/year. The input is not driving the schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>and the two disagree by $504,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Net effect: nobody could have read a correct CPA, ROI, or total spend figure out of this model at any point in 2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A14:J14"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B8:I9">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="4">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7867,7 +8469,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -7980,7 +8581,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>

</xml_diff>